<commit_message>
feat: release-check 리비전 비교 추가 (v3.7.0)
- compare_revisions.py: 브랜치·리비전 diff 컨텍스트 생성
- branch-merge-base, branch-tip, revision, revision-merge-base 모드
- 엑셀 요약에 비교 방식·비교 기준·merge-base 표시
- 샘플 JSON·xlsx와 문서 갱신
</commit_message>
<xml_diff>
--- a/samples/release-check/release-check-sample.xlsx
+++ b/samples/release-check/release-check-sample.xlsx
@@ -537,7 +537,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>릴리스 전 브랜치 diff 점검 보고서</t>
+          <t>릴리스 전 diff 점검 보고서</t>
         </is>
       </c>
     </row>
@@ -568,78 +568,90 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>비교 브랜치</t>
+          <t>비교 방식</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>main → develop</t>
+          <t>브랜치 merge-base</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>merge-base</t>
+          <t>비교 기준</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>a1b2c3d4</t>
+          <t>main → develop</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>생성 시각</t>
+          <t>merge-base</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-27T11:00:00+09:00</t>
+          <t>a1b2c3d4</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>커밋 수</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>7</v>
+          <t>생성 시각</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-10-27T11:00:00+09:00</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>변경 파일 수</t>
+          <t>커밋 수</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>증감 라인</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>+340 / -85</t>
-        </is>
+          <t>변경 파일 수</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>증감 라인</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>+340 / -85</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>점검 항목</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B12" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: release-check 역할 컬럼·비개발자 문장 추가 (v3.8.0)
- 점검 항목에 역할 컬럼 추가 (ADMIN → 관리자)
- 점검 항목·기대 결과를 비개발자 관점 문장으로 작성
- 엑셀에서 변경 근거 열 제거, 기술 근거는 JSON에 보관
- 샘플 JSON·xlsx 갱신
</commit_message>
<xml_diff>
--- a/samples/release-check/release-check-sample.xlsx
+++ b/samples/release-check/release-check-sample.xlsx
@@ -835,10 +835,10 @@
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
@@ -859,22 +859,22 @@
       </c>
       <c r="C1" s="12" t="inlineStr">
         <is>
+          <t>역할</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
           <t>영역</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="E1" s="12" t="inlineStr">
         <is>
           <t>점검 항목</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>기대 결과</t>
-        </is>
-      </c>
-      <c r="F1" s="12" t="inlineStr">
-        <is>
-          <t>변경 근거</t>
         </is>
       </c>
       <c r="G1" s="12" t="inlineStr">
@@ -916,22 +916,22 @@
       </c>
       <c r="C2" s="15" t="inlineStr">
         <is>
+          <t>보안</t>
+        </is>
+      </c>
+      <c r="D2" s="15" t="inlineStr">
+        <is>
           <t>인증</t>
         </is>
       </c>
-      <c r="D2" s="15" t="inlineStr">
-        <is>
-          <t>비밀번호 재설정 링크가 24시간 후 만료되는지 확인</t>
-        </is>
-      </c>
       <c r="E2" s="15" t="inlineStr">
         <is>
-          <t>만료 후 접근 시 오류 메시지 표시</t>
+          <t>비밀번호 재설정 링크가 하루가 지나면 더 이상 동작하지 않는지 확인</t>
         </is>
       </c>
       <c r="F2" s="15" t="inlineStr">
         <is>
-          <t>src/auth/reset.js (9f8e7d6)</t>
+          <t>24시간 후 링크를 열면 만료 안내가 표시되고 비밀번호를 바꿀 수 없음</t>
         </is>
       </c>
       <c r="G2" s="15" t="inlineStr">
@@ -961,22 +961,22 @@
       </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
+          <t>관리자</t>
+        </is>
+      </c>
+      <c r="D3" s="15" t="inlineStr">
+        <is>
           <t>API</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
-        <is>
-          <t>공유 API 호출 시 권한 없는 사용자가 403을 받는지 확인</t>
-        </is>
-      </c>
       <c r="E3" s="15" t="inlineStr">
         <is>
-          <t>403과 오류 코드 반환</t>
+          <t>권한 없는 사용자가 공유 기능에 접근하면 차단되는지 확인</t>
         </is>
       </c>
       <c r="F3" s="15" t="inlineStr">
         <is>
-          <t>src/api/share.js (7c6b5a4)</t>
+          <t>접근이 차단되고 ‘권한이 없습니다’ 안내가 표시됨</t>
         </is>
       </c>
       <c r="G3" s="15" t="inlineStr">
@@ -1006,22 +1006,22 @@
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
+          <t>PM</t>
+        </is>
+      </c>
+      <c r="D4" s="15" t="inlineStr">
+        <is>
           <t>문서</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
-        <is>
-          <t>README의 공유 기능 설명이 실제 동작과 일치하는지 확인</t>
-        </is>
-      </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>설명대로 동작</t>
+          <t>사용 안내에 적힌 공유 기능 설명이 실제 화면과 같은지 확인</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>README.md</t>
+          <t>안내를 따라 했을 때 화면과 동작이 설명과 일치함</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
@@ -1068,22 +1068,22 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
           <t>DB</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
-        <is>
-          <t>공유 테이블 마이그레이션이 기존 데이터와 충돌하지 않는지 확인</t>
-        </is>
-      </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>마이그레이션 롤백 후 재적용 시 오류 없음</t>
+          <t>새 공유 기능을 배포해도 기존 예약 데이터가 깨지지 않는지 확인</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>db/migrations/0042_share.sql (3d2c1b0)</t>
+          <t>배포 후 기존 예약과 사용자 데이터가 그대로 보이고, 공유 기능을 켜도 오류가 나지 않음</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -1113,22 +1113,22 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
           <t>인증</t>
         </is>
       </c>
-      <c r="D7" s="15" t="inlineStr">
-        <is>
-          <t>토큰 만료 검증이 서버 시간 기준인지 코드 확인</t>
-        </is>
-      </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>클라이언트 시간 조작으로 우회 불가</t>
+          <t>사용자 기기 시간을 바꿔도 로그인 만료가 우회되지 않는지 확인</t>
         </is>
       </c>
       <c r="F7" s="15" t="inlineStr">
         <is>
-          <t>src/auth/reset.js (9f8e7d6)</t>
+          <t>기기 시간을 바꿔도 만료된 로그인은 다시 사용할 수 없음</t>
         </is>
       </c>
       <c r="G7" s="15" t="inlineStr">
@@ -1158,22 +1158,22 @@
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
+          <t>개발</t>
+        </is>
+      </c>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
           <t>API</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
-        <is>
-          <t>공유 API의 트랜잭션 경계가 중복 생성을 막는지 코드 확인</t>
-        </is>
-      </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>동시 요청에서도 1건만 생성</t>
+          <t>같은 공유 요청이 동시에 두 번 들어와도 공유가 한 번만 만들어지는지 확인</t>
         </is>
       </c>
       <c r="F8" s="15" t="inlineStr">
         <is>
-          <t>src/api/share.js (7c6b5a4)</t>
+          <t>동시에 두 번 요청해도 공유 항목은 1개만 생성됨</t>
         </is>
       </c>
       <c r="G8" s="15" t="inlineStr">
@@ -1194,12 +1194,15 @@
   <mergeCells count="1">
     <mergeCell ref="A5:K5"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="3">
     <dataValidation sqref="B2:B4 B6:B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"P0,P1,P2"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H4 H6:H8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"미확인,통과,실패,해당 없음"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C4 C6:C8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ADMIN,PM,QA,DEV,OPS,SEC,DATA,DESIGN,ETC,UNASSIGNED"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>